<commit_message>
added escape barrier score info
</commit_message>
<xml_diff>
--- a/Escape Barrier Analysis/escape barrier score/data/Path Frequencies.xlsx
+++ b/Escape Barrier Analysis/escape barrier score/data/Path Frequencies.xlsx
@@ -5,16 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anitido/Documents/GitHub/Escapability/Escape Barrier Data and Analysis/escape barrier score/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anitido/Documents/GitHub/Escapability/Escape Barrier Analysis/escape barrier score/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B9CE35E-D4F8-0D4F-9150-1EE978622AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB255F8-84D1-C149-A1BE-FFA55E3132E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28440" yWindow="2880" windowWidth="39980" windowHeight="20340" xr2:uid="{475633B7-6B96-0B42-840E-0F2F194B55BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Samples" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$1</definedName>
@@ -93,16 +92,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -155,22 +146,19 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,359 +483,359 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="4" t="str">
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="str">
         <f t="shared" ref="E2:E17" si="0">_xlfn.CONCAT(B2,"-",C2,"-",D2)</f>
         <v>REJOc-VRC07-A</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>0.6470588235294118</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="4" t="str">
+      <c r="C3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc-VRC07-B</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <v>0.35294117647058826</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="4" t="str">
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc-N6-A</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>0.58823529411764708</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="4" t="str">
+      <c r="D5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc-N6-B</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>0.41176470588235292</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E6" s="4" t="str">
+      <c r="D6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc-PGDM1400-A</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="4">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="3">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="4" t="str">
+      <c r="D7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc-PGDM1400-B</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>0.44</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="3">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E8" s="4" t="str">
+      <c r="C8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="3" t="str">
         <f t="shared" si="0"/>
         <v>JRCSF-VRC07-A</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <v>0.6428571428571429</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="4">
-        <v>4</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="3">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E9" s="4" t="str">
+      <c r="C9" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="3" t="str">
         <f t="shared" si="0"/>
         <v>JRCSF-VRC07-B</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <v>0.35714285714285715</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="4">
-        <v>5</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="3">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E10" s="4" t="str">
+      <c r="C10" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="3" t="str">
         <f t="shared" si="0"/>
         <v>RV-VRC07-A</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <v>0.55555555555555558</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="4">
-        <v>5</v>
-      </c>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="3">
+        <v>5</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" s="4" t="str">
+      <c r="C11" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="3" t="str">
         <f t="shared" si="0"/>
         <v>RV-VRC07-B</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="4">
-        <v>5</v>
-      </c>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="3">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="4" t="str">
+      <c r="E12" s="3" t="str">
         <f t="shared" si="0"/>
         <v>RV-VRC07-C</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="5">
         <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E13" s="4" t="str">
+      <c r="C13" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc+M184I/V-VRC07-A</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <v>0.59</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>6</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" s="4" t="str">
+      <c r="C14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="3" t="str">
         <f t="shared" si="0"/>
         <v>REJOc+M184I/V-VRC07-B</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <v>0.41</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>7</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E15" s="4" t="str">
+      <c r="D15" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="3" t="str">
         <f t="shared" si="0"/>
         <v>JRCSF-N6-A</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>8</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E16" s="4" t="str">
+      <c r="D16" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="3" t="str">
         <f t="shared" si="0"/>
         <v>JRCSF-PGDM1400-A</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="4">
         <v>0.33</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="4">
+      <c r="A17" s="3">
         <v>8</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="4" t="str">
+      <c r="D17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="3" t="str">
         <f t="shared" si="0"/>
         <v>JRCSF-PGDM1400-B</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="4">
         <v>0.67</v>
       </c>
     </row>
@@ -855,20 +843,4 @@
   <autoFilter ref="A1:G1" xr:uid="{747A8BA9-5EB5-7442-9D54-7FF11E90551F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3393BDD-1D8D-0448-A94B-CF342A786B23}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>